<commit_message>
feat: implement batch analysis dashboard
</commit_message>
<xml_diff>
--- a/reports/summary.xlsx
+++ b/reports/summary.xlsx
@@ -417,13 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -457,23 +457,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Amit Kumar</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Strongly Recommend</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Python, SQL, Git, Flask</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Rahul Sharma</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>87</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Strongly Recommend</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Python, SQL, Flask</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Git</t>
         </is>

</xml_diff>